<commit_message>
Fix #362/#363 bundling error; sync roadmap with #7/#515/#362 completion
ROADMAP.md's "Full execution order" incorrectly bundled #363 into #362's
stated M0 chain. #363 actually depends on #350/#448 (not yet built) and
is flagged in its own issue body as a likely duplicate that folds into
#350's runtime envelopes + #448's engine commands/events rather than
being implemented standalone. Moves #363 to the unordered "remaining M0
issues" list with its real dependency and duplicate-candidate status
noted.

Also brings the roadmap current with work merged since this branch was
first drafted: #7 (CI pipeline), #515 (architecture-boundary guard), and
#362 (canonical domain model) are now closed; #314 is the next M0 chain
step. Regenerates scripts/roadmap-data.json and the workbook/previews to
match.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/roadmap-visual/bible-challenge-roadmap.xlsx
+++ b/outputs/roadmap-visual/bible-challenge-roadmap.xlsx
@@ -1520,7 +1520,7 @@
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>In progress (#7/#515/#362 done; #314 next)</t>
         </is>
       </c>
       <c r="F14" s="21" t="inlineStr"/>
@@ -2549,7 +2549,7 @@
         </is>
       </c>
       <c r="C38" s="38" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D38" s="1" t="n"/>
       <c r="E38" s="1" t="n"/>
@@ -5340,7 +5340,7 @@
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F9" s="9" t="inlineStr">
@@ -5350,7 +5350,7 @@
       </c>
       <c r="G9" s="10" t="inlineStr">
         <is>
-          <t>Do first</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H9" s="1" t="n"/>
@@ -5371,12 +5371,12 @@
       <c r="A10" s="1" t="n"/>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>#362, #314, #447-#450</t>
+          <t>#362</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Domain model, GameDefinition registry, Engine SDK</t>
+          <t>Canonical domain model, stable IDs, ownership boundaries</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
@@ -5386,17 +5386,17 @@
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>#362 -&gt; #314 -&gt; #447</t>
+          <t>None</t>
         </is>
       </c>
       <c r="G10" s="10" t="inlineStr">
         <is>
-          <t>Foundation core</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H10" s="1" t="n"/>
@@ -5417,12 +5417,12 @@
       <c r="A11" s="1" t="n"/>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>#350, #448, #351, #353</t>
+          <t>#314, #447-#450</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>Intents/events, projections, session persistence</t>
+          <t>GameDefinition registry, Engine SDK</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
@@ -5437,12 +5437,12 @@
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>#349, #350</t>
+          <t>#362 (done) -&gt; #314 -&gt; #447</t>
         </is>
       </c>
       <c r="G11" s="10" t="inlineStr">
         <is>
-          <t>Foundation core</t>
+          <t>Foundation core, next</t>
         </is>
       </c>
       <c r="H11" s="1" t="n"/>
@@ -5463,12 +5463,12 @@
       <c r="A12" s="1" t="n"/>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>#513, #514, #519</t>
+          <t>#350, #448, #351, #353</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>LegacyGameAdapter, Offline adapter, local security baseline</t>
+          <t>Intents/events, projections, session persistence</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
@@ -5483,12 +5483,12 @@
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>#314; #349</t>
+          <t>#349, #350</t>
         </is>
       </c>
       <c r="G12" s="10" t="inlineStr">
         <is>
-          <t>M0 exit items</t>
+          <t>Foundation core</t>
         </is>
       </c>
       <c r="H12" s="1" t="n"/>
@@ -5509,12 +5509,12 @@
       <c r="A13" s="1" t="n"/>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>#522, #523, #524</t>
+          <t>#513, #514, #519</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>Gameplay lifecycle/resolution policies, gameplay shell/viewport contract, cross-game scoring normalization</t>
+          <t>LegacyGameAdapter, Offline adapter, local security baseline</t>
         </is>
       </c>
       <c r="D13" s="9" t="inlineStr">
@@ -5529,12 +5529,12 @@
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t>#509; #524 coordinates with #364</t>
+          <t>#314; #349</t>
         </is>
       </c>
       <c r="G13" s="10" t="inlineStr">
         <is>
-          <t>M0 exit gate — required before #510 begins; kept as three distinct issues (behavior, layout, scoring)</t>
+          <t>M0 exit items</t>
         </is>
       </c>
       <c r="H13" s="1" t="n"/>
@@ -5555,17 +5555,17 @@
       <c r="A14" s="1" t="n"/>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>#510</t>
+          <t>#522, #523, #524</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>Five Clues reference migration</t>
+          <t>Gameplay lifecycle/resolution policies, gameplay shell/viewport contract, cross-game scoring normalization</t>
         </is>
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>M0</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -5575,12 +5575,12 @@
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>#509, #402, #4, #516, #522, #523, #524</t>
+          <t>#509; #524 coordinates with #364</t>
         </is>
       </c>
       <c r="G14" s="10" t="inlineStr">
         <is>
-          <t>Proof gate; proves #522/#523/#524, does not itself define the cross-game scoring scale</t>
+          <t>M0 exit gate — required before #510 begins; kept as three distinct issues (behavior, layout, scoring)</t>
         </is>
       </c>
       <c r="H14" s="1" t="n"/>
@@ -5601,12 +5601,12 @@
       <c r="A15" s="1" t="n"/>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>#402, #4, #516</t>
+          <t>#510</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>Answer evaluation, oracle tests, vNext surface host</t>
+          <t>Five Clues reference migration</t>
         </is>
       </c>
       <c r="D15" s="9" t="inlineStr">
@@ -5621,12 +5621,12 @@
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>#350, #338; #314, #351</t>
+          <t>#509, #402, #4, #516, #522, #523, #524</t>
         </is>
       </c>
       <c r="G15" s="10" t="inlineStr">
         <is>
-          <t>M1 prerequisites</t>
+          <t>Proof gate; proves #522/#523/#524, does not itself define the cross-game scoring scale</t>
         </is>
       </c>
       <c r="H15" s="1" t="n"/>
@@ -5647,17 +5647,17 @@
       <c r="A16" s="1" t="n"/>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>#507</t>
+          <t>#402, #4, #516</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>Audience-boundary catalog audit</t>
+          <t>Answer evaluation, oracle tests, vNext surface host</t>
         </is>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -5667,12 +5667,12 @@
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>None (root)</t>
+          <t>#350, #338; #314, #351</t>
         </is>
       </c>
       <c r="G16" s="10" t="inlineStr">
         <is>
-          <t>Parallel now</t>
+          <t>M1 prerequisites</t>
         </is>
       </c>
       <c r="H16" s="1" t="n"/>
@@ -5693,12 +5693,12 @@
       <c r="A17" s="1" t="n"/>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>#511</t>
+          <t>#507</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>Migration-wave classification</t>
+          <t>Audience-boundary catalog audit</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
@@ -5713,12 +5713,12 @@
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
-          <t>#507, #510</t>
+          <t>None (root)</t>
         </is>
       </c>
       <c r="G17" s="10" t="inlineStr">
         <is>
-          <t>After M1</t>
+          <t>Parallel now</t>
         </is>
       </c>
       <c r="H17" s="1" t="n"/>
@@ -5739,17 +5739,17 @@
       <c r="A18" s="1" t="n"/>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>#331, #305-#309</t>
+          <t>#511</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>Migration waves epic + wave placeholders</t>
+          <t>Migration-wave classification</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M2</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -5759,12 +5759,12 @@
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>#511</t>
+          <t>#507, #510</t>
         </is>
       </c>
       <c r="G18" s="10" t="inlineStr">
         <is>
-          <t>Scope from #511</t>
+          <t>After M1</t>
         </is>
       </c>
       <c r="H18" s="1" t="n"/>
@@ -5785,12 +5785,12 @@
       <c r="A19" s="1" t="n"/>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>#56-#58, #87</t>
+          <t>#331, #305-#309</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>Legacy variants (timeline, Director's Cut, Word Ladder)</t>
+          <t>Migration waves epic + wave placeholders</t>
         </is>
       </c>
       <c r="D19" s="9" t="inlineStr">
@@ -5805,12 +5805,12 @@
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>Owning wave</t>
+          <t>#511</t>
         </is>
       </c>
       <c r="G19" s="10" t="inlineStr">
         <is>
-          <t>Do not implement yet</t>
+          <t>Scope from #511</t>
         </is>
       </c>
       <c r="H19" s="1" t="n"/>
@@ -5831,17 +5831,17 @@
       <c r="A20" s="1" t="n"/>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>#11-#20, #50-#51</t>
+          <t>#56-#58, #87</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>Phone Mode (folded into M6)</t>
+          <t>Legacy variants (timeline, Director's Cut, Word Ladder)</t>
         </is>
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>M6</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -5851,7 +5851,7 @@
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
-          <t>#510, #350, #351</t>
+          <t>Owning wave</t>
         </is>
       </c>
       <c r="G20" s="10" t="inlineStr">
@@ -5877,17 +5877,17 @@
       <c r="A21" s="1" t="n"/>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>#103, #105-#108</t>
+          <t>#11-#20, #50-#51</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>Agon UI redesign as vNext surfaces</t>
+          <t>Phone Mode (folded into M6)</t>
         </is>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M6</t>
         </is>
       </c>
       <c r="E21" s="9" t="inlineStr">
@@ -5897,7 +5897,7 @@
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>#510, #516</t>
+          <t>#510, #350, #351</t>
         </is>
       </c>
       <c r="G21" s="10" t="inlineStr">
@@ -5923,17 +5923,17 @@
       <c r="A22" s="1" t="n"/>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>#99-#102, #117</t>
+          <t>#103, #105-#108</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>Brand &amp; design system</t>
+          <t>Agon UI redesign as vNext surfaces</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>Track</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -5943,12 +5943,12 @@
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>#117 -&gt; #99 -&gt; #100 -&gt; #101 -&gt; #102</t>
+          <t>#510, #516</t>
         </is>
       </c>
       <c r="G22" s="10" t="inlineStr">
         <is>
-          <t>Parallel now</t>
+          <t>Do not implement yet</t>
         </is>
       </c>
       <c r="H22" s="1" t="n"/>
@@ -5969,17 +5969,17 @@
       <c r="A23" s="1" t="n"/>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>#15</t>
+          <t>#99-#102, #117</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>1.0.0 stabilization (Local vNext)</t>
+          <t>Brand &amp; design system</t>
         </is>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>1.0.0</t>
+          <t>Track</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
@@ -5989,12 +5989,12 @@
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>#509, #510, #353, #357, #7, #305-#308, UI</t>
+          <t>#117 -&gt; #99 -&gt; #100 -&gt; #101 -&gt; #102</t>
         </is>
       </c>
       <c r="G23" s="10" t="inlineStr">
         <is>
-          <t>Release gate</t>
+          <t>Parallel now</t>
         </is>
       </c>
       <c r="H23" s="1" t="n"/>
@@ -6015,17 +6015,17 @@
       <c r="A24" s="1" t="n"/>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>#189-#198, #310</t>
+          <t>#15</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>Tournaments &amp; persistent events</t>
+          <t>1.0.0 stabilization (Local vNext)</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>Track</t>
+          <t>1.0.0</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -6035,12 +6035,12 @@
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>#314, #353, #364; #191/#194 also need #524; #197/#310 need M4</t>
+          <t>#509, #510, #353, #357, #7, #305-#308, UI</t>
         </is>
       </c>
       <c r="G24" s="10" t="inlineStr">
         <is>
-          <t>After M0; #197/#310 after M4</t>
+          <t>Release gate</t>
         </is>
       </c>
       <c r="H24" s="1" t="n"/>
@@ -6061,17 +6061,17 @@
       <c r="A25" s="1" t="n"/>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>#130-#169, #280-#285</t>
+          <t>#189-#198, #310</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>Cards, randomizers, timer, image board</t>
+          <t>Tournaments &amp; persistent events</t>
         </is>
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>Track</t>
         </is>
       </c>
       <c r="E25" s="9" t="inlineStr">
@@ -6081,12 +6081,12 @@
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>#447, #142, #156</t>
+          <t>#314, #353, #364; #191/#194 also need #524; #197/#310 need M4</t>
         </is>
       </c>
       <c r="G25" s="10" t="inlineStr">
         <is>
-          <t>After M0</t>
+          <t>After M0; #197/#310 after M4</t>
         </is>
       </c>
       <c r="H25" s="1" t="n"/>
@@ -6107,17 +6107,17 @@
       <c r="A26" s="1" t="n"/>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>M7 games</t>
+          <t>#130-#169, #280-#285</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>Pairs of Faith, Wayfinder, Multitude, Baseball, ...</t>
+          <t>Cards, randomizers, timer, image board</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>M7</t>
+          <t>M3</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -6127,12 +6127,12 @@
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>#509 + capability + #507</t>
+          <t>#447, #142, #156</t>
         </is>
       </c>
       <c r="G26" s="10" t="inlineStr">
         <is>
-          <t>Do not implement yet</t>
+          <t>After M0</t>
         </is>
       </c>
       <c r="H26" s="1" t="n"/>
@@ -6153,17 +6153,17 @@
       <c r="A27" s="1" t="n"/>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>M8 games</t>
+          <t>M7 games</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>Kids games, Journeys, Activity Events</t>
+          <t>Pairs of Faith, Wayfinder, Multitude, Baseball, ...</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>M8</t>
+          <t>M7</t>
         </is>
       </c>
       <c r="E27" s="9" t="inlineStr">
@@ -6173,7 +6173,7 @@
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>#234 + capability</t>
+          <t>#509 + capability + #507</t>
         </is>
       </c>
       <c r="G27" s="10" t="inlineStr">
@@ -6199,17 +6199,17 @@
       <c r="A28" s="1" t="n"/>
       <c r="B28" s="8" t="inlineStr">
         <is>
-          <t>#359, #360, #377, #378</t>
+          <t>M8 games</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>Shared/Hosted runtimes and Stage adapters</t>
+          <t>Kids games, Journeys, Activity Events</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>M9</t>
+          <t>M8</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -6219,12 +6219,12 @@
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>#357 and M6 contracts</t>
+          <t>#234 + capability</t>
         </is>
       </c>
       <c r="G28" s="10" t="inlineStr">
         <is>
-          <t>Future</t>
+          <t>Do not implement yet</t>
         </is>
       </c>
       <c r="H28" s="1" t="n"/>
@@ -6245,17 +6245,17 @@
       <c r="A29" s="1" t="n"/>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>#517</t>
+          <t>#359, #360, #377, #378</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>Legacy retirement epic</t>
+          <t>Shared/Hosted runtimes and Stage adapters</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>M10</t>
+          <t>M9</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
@@ -6265,12 +6265,12 @@
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>#331</t>
+          <t>#357 and M6 contracts</t>
         </is>
       </c>
       <c r="G29" s="10" t="inlineStr">
         <is>
-          <t>Last</t>
+          <t>Future</t>
         </is>
       </c>
       <c r="H29" s="1" t="n"/>
@@ -6289,34 +6289,34 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n"/>
-      <c r="B30" s="11" t="inlineStr">
-        <is>
-          <t>#23/#286, #243/#484, #304, #321, #363, ...</t>
-        </is>
-      </c>
-      <c r="C30" s="12" t="inlineStr">
-        <is>
-          <t>Duplicate candidates (phase 7)</t>
-        </is>
-      </c>
-      <c r="D30" s="12" t="inlineStr">
-        <is>
-          <t>Various</t>
-        </is>
-      </c>
-      <c r="E30" s="12" t="inlineStr">
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>#517</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>Legacy retirement epic</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="F30" s="12" t="inlineStr">
-        <is>
-          <t>Requirements migration</t>
-        </is>
-      </c>
-      <c r="G30" s="13" t="inlineStr">
-        <is>
-          <t>Do not close without approval</t>
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t>#331</t>
+        </is>
+      </c>
+      <c r="G30" s="10" t="inlineStr">
+        <is>
+          <t>Last</t>
         </is>
       </c>
       <c r="H30" s="1" t="n"/>
@@ -6335,12 +6335,36 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n"/>
-      <c r="B31" s="1" t="n"/>
-      <c r="C31" s="1" t="n"/>
-      <c r="D31" s="1" t="n"/>
-      <c r="E31" s="1" t="n"/>
-      <c r="F31" s="1" t="n"/>
-      <c r="G31" s="1" t="n"/>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>#23/#286, #243/#484, #304, #321, #363, ...</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>Duplicate candidates (phase 7)</t>
+        </is>
+      </c>
+      <c r="D31" s="12" t="inlineStr">
+        <is>
+          <t>Various</t>
+        </is>
+      </c>
+      <c r="E31" s="12" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F31" s="12" t="inlineStr">
+        <is>
+          <t>Requirements migration</t>
+        </is>
+      </c>
+      <c r="G31" s="13" t="inlineStr">
+        <is>
+          <t>Do not close without approval</t>
+        </is>
+      </c>
       <c r="H31" s="1" t="n"/>
       <c r="I31" s="1" t="n"/>
       <c r="J31" s="1" t="n"/>
@@ -7328,10 +7352,10 @@
         <v>1</v>
       </c>
       <c r="G9" s="15" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I9" s="9" t="inlineStr">
         <is>

</xml_diff>